<commit_message>
Sync the production workbook to Scene 1 and Scenes 1–21.
Match the Hisaab Kitaab opening, AnuKool and PratiKool, and the timing column.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/navarasa-master-production.xlsx
+++ b/docs/navarasa-master-production.xlsx
@@ -475,13 +475,15 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Master production workbook — cleaned copy (Scenes 1–15 locked; 16–19 prior draft)</t>
-        </is>
-      </c>
-    </row>
+          <t>Master production workbook — Scenes 1–21. Scene 1 timing TBD; Scenes 2–21 ≈95 min.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -499,7 +501,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2. Scene Overview — all 19 scenes at a glance</t>
+          <t>2. Scene Overview — all 21 scenes at a glance (includes Timing column)</t>
         </is>
       </c>
     </row>
@@ -531,6 +533,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
@@ -638,17 +641,17 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Cool</t>
+          <t>AnuKool</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Anukool (was Kool)</t>
+          <t>was Kool / Cool</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Light shadow — cheerful, optimistic, supportive; amplifies resilience</t>
+          <t>Bright shadow — optimistic, encouraging; Very Cool boy</t>
         </is>
       </c>
     </row>
@@ -660,17 +663,17 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Pratikool</t>
+          <t>PratiKool</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>PratiKool</t>
+          <t>was Pratikool</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Dark shadow — gruff, cynical, disruptive; instigates jealousy and conflict</t>
+          <t>Dark shadow — cynical, provocative; Bad boy</t>
         </is>
       </c>
     </row>
@@ -977,7 +980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1043,6 +1046,11 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Timing (min)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
@@ -1055,7 +1063,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>The Cosmic Handover</t>
+          <t>Karma Operations – The Hisaab Kitaab Department</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -1070,27 +1078,32 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Startup lab → stage → Karma Chakra</t>
+          <t>Karma Operations (heaven) → Earth tech hub → chariot</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>AKV, Maya, Karma, Cool, Pratikool</t>
+          <t>Karma Dev, AnuKool, PratiKool, AKV, Maya</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Electronic entrance + Navras/Karma Chakra title anthem</t>
+          <t>Ethereal welcome · कर्म entrance · Maya theme · NAVARASA title</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>AKV gifts Maya; Navarasas plan; chariot ascent</t>
+          <t>Welcome + shadow sprint → overload → swipe to AKV → Maya has no emotions → title song home</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Locked</t>
+          <t>Draft — dialogue locked</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
     </row>
@@ -1125,7 +1138,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Karma, Cool, Pratikool, Maya</t>
+          <t>Karma, AnuKool, PratiKool, Maya</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -1142,6 +1155,9 @@
         <is>
           <t>Locked</t>
         </is>
+      </c>
+      <c r="K3" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -1193,6 +1209,9 @@
           <t>Locked</t>
         </is>
       </c>
+      <c r="K4" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -1225,7 +1244,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Karma, Cool, Pratikool, Maya</t>
+          <t>Karma, AnuKool, PratiKool, Maya</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -1242,6 +1261,9 @@
         <is>
           <t>Locked</t>
         </is>
+      </c>
+      <c r="K5" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -1293,6 +1315,9 @@
           <t>Locked</t>
         </is>
       </c>
+      <c r="K6" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -1343,6 +1368,9 @@
           <t>Locked</t>
         </is>
       </c>
+      <c r="K7" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -1393,55 +1421,61 @@
           <t>Locked</t>
         </is>
       </c>
+      <c r="K8" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>III Fracturing</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Celestial Infiltration</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Screen → Stage</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>II Earthly Arena</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Song Continuation on Stage</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Heavens → Earth training camp</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Karma, Cool, Pratikool</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Descent AI graphic</t>
-        </is>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>Karma: real plot found; shadows descend</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>Locked</t>
-        </is>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Stage — song coda</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Karan, Arjun</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Song last para / coda TBD</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Karan song coda; Arjun focus/Walia threat; Satak joke; both laugh</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1455,12 +1489,12 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Sowing Seeds of Paranoia</t>
+          <t>Celestial Infiltration</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>Screen → Stage</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -1470,28 +1504,31 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Satak Singh's camp</t>
+          <t>Heavens → Earth training camp</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Cool, Pratikool, Coach Satak Singh</t>
+          <t>Karma, AnuKool, PratiKool</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Comic/dark sting</t>
+          <t>Descent AI graphic</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Spies pitch; Satak absorbs them into camp</t>
+          <t>Karma: real plot found; shadows descend</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
           <t>Locked</t>
         </is>
+      </c>
+      <c r="K10" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -1505,7 +1542,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>The Gym – The Silent Sting</t>
+          <t>Sowing Seeds of Paranoia</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1520,28 +1557,31 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Athletic training facility</t>
+          <t>Satak Singh's camp</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Karan, Satak, Arjun, Cool, Pratikool, friends</t>
+          <t>AnuKool, PratiKool, Coach Satak Singh</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Training underscore</t>
+          <t>Comic/dark sting</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Arjun showboats/insults; Pratikool stokes; Coach worried; Cool pitches marketing party</t>
+          <t>Spies pitch; Satak absorbs them into camp</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
           <t>Locked</t>
         </is>
+      </c>
+      <c r="K11" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -1555,143 +1595,152 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
+          <t>The Gym – The Silent Sting</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Athletic training facility</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Karan, Satak, Arjun, AnuKool, PratiKool, friends</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Training underscore</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Arjun showboats/insults; PratiKool stokes; Coach worried; AnuKool pitches marketing party</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>III Fracturing</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
           <t>Karma Operations Centre – Twist &amp; Hasya Setup</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Video / Stage</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Hasya (setup)</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Celestial Karma Operations Center</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Karma Dev, Maya</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Hasya Sanskrit shloka</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>Maya asks friendship twist; Karma teaches Hasya; sings Hasya shloka → marketing event</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
         <is>
           <t>Locked</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" t="inlineStr">
+      <c r="K13" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>III Fracturing</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Hasya Ras – Marketing Pre-Event Qawwali Party</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Hasya</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Race marketing pre-event party stage</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Ruchi, Arjun, Karan, friends, Cool, Pratikool, ensemble</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Ruchi, Arjun, Karan, friends, AnuKool, PratiKool, ensemble</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>Qawwali · Oiyamma · Sharara · Ghaghra · Dhurandhar</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Cool's party plan; Ruchi hosts; Arjun qawwali + medley</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>AnuKool's party plan; Ruchi hosts; Arjun qawwali + medley</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>Draft</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>III Fracturing</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Raudra Ras – Stage Crash &amp; Birth of a Rival</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>Raudra</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Marketing party stage → crashed</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Arjun, Karan, Sports Crew, Pratikool, Karma</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Mary and Me; Malhari; Raudra shloka</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>Malhari clash mid-party; Arjun vows sporting war</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>Locked</t>
-        </is>
+      <c r="K14" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="15">
@@ -1700,48 +1749,51 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>IV Fall &amp; Resurgence</t>
+          <t>III Fracturing</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>The Sabotage &amp; The Fall</t>
+          <t>Raudra Ras – Stage Crash &amp; Birth of a Rival</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Stage</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Bibhatsa / tragedy lead-in</t>
+          <t>Raudra</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Open training highway</t>
+          <t>Marketing party stage → crashed</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Karan, Arjun's crew, Karma</t>
+          <t>Arjun, Karan, Sports Crew, PratiKool, Karma</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Uplifting ride → crash → mourning shloka</t>
+          <t>Mary and Me; Malhari; Raudra shloka</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Invisible wire trap; cycle destroyed; Karan down</t>
+          <t>Malhari clash mid-party; Arjun vows sporting war</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
           <t>Locked</t>
         </is>
+      </c>
+      <c r="K15" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -1755,43 +1807,46 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Karuna Ras – The Shattered Dream</t>
+          <t>The Sabotage &amp; The Fall</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Video / Stage</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Karuna</t>
+          <t>Bibhatsa / tragedy lead-in</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Hospital room / corridor</t>
+          <t>Open training highway</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Karan, Satak, Ajay Walia (phone), Karma, Maya</t>
+          <t>Karan, Arjun's crew, Karma</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Karuna theme + shloka</t>
+          <t>Uplifting ride → crash → mourning shloka</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Sponsorship cancelled; contract torn over bed</t>
+          <t>Invisible wire trap; cycle destroyed; Karan down</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
           <t>Locked</t>
         </is>
+      </c>
+      <c r="K16" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -1805,43 +1860,46 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>The Comeback Ignition</t>
+          <t>Karuna Ras – The Shattered Dream</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Stage → Montage</t>
+          <t>Video / Stage</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Veer (inner valor)</t>
+          <t>Karuna</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Recovery → workshop → track</t>
+          <t>Hospital room / corridor</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Karan, Cool, Brishti, Gaurav, Anu, Shikha, Shri</t>
+          <t>Karan, Satak, Ajay Walia (phone), Karma, Maya</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Comeback anthem</t>
+          <t>Karuna theme + shloka</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Rage held; friends assign roles; physio + bike rebuild montage</t>
+          <t>Sponsorship cancelled; contract torn over bed</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
           <t>Locked</t>
         </is>
+      </c>
+      <c r="K17" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -1850,48 +1908,51 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>V Race (prior draft)</t>
+          <t>IV Fall &amp; Resurgence</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Cycle Race &amp; Final 3 Laps</t>
+          <t>The Comeback Ignition</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Video / Stage</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Stage → Montage</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Veer (inner valor)</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Start → road → VIP → stadium</t>
+          <t>Recovery → workshop → track</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Karan, Arjun, Walia, Satak, crowd, Cool, Pratikool, Karma, Maya</t>
+          <t>Karan, AnuKool, Brishti, Gaurav, Anu, Shikha, Shri</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>Race fanfare</t>
+          <t>Comeback anthem</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Karan returns; duel; FINAL 3 LAPS</t>
+          <t>Rage held; friends assign roles; physio + bike rebuild montage</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>Prior draft — polish TBD</t>
-        </is>
+          <t>Locked</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="19">
@@ -1905,43 +1966,46 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Adbhuta Ras – Sacrifice &amp; Choice</t>
+          <t>Cycle Race &amp; Final 3 Laps</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Video → Stage</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>Adbhuta</t>
+          <t>Video / Stage</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Track → heaven</t>
+          <t>Start → road → VIP → stadium</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Karan, Arjun, Maya, Karma, Pratikool</t>
+          <t>Karan, Arjun, Walia, Satak, crowd, AnuKool, PratiKool, Karma, Maya</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Adbhuta swell</t>
+          <t>Race fanfare</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Chain snaps; Arjun gives bike; humans have Choice</t>
+          <t>Karan returns; duel; FINAL 3 LAPS</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
           <t>Prior draft — polish TBD</t>
         </is>
+      </c>
+      <c r="K19" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -1950,48 +2014,51 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>VI Coda (prior draft)</t>
+          <t>V Race (prior draft)</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Bhayanaka Ras – Raktabija &amp; Mahakali</t>
+          <t>Adbhuta Ras – Sacrifice &amp; Choice</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Stage / Video</t>
+          <t>Video → Stage</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Bhayanaka</t>
+          <t>Adbhuta</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Cosmic battlefield</t>
+          <t>Track → heaven</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Karma, Maya, Raktabija, Maa Kali</t>
+          <t>Karan, Arjun, Maya, Karma, PratiKool</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Tandava</t>
+          <t>Adbhuta swell</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Blood-demon myth → Kali Tandava</t>
+          <t>Chain snaps; Arjun gives bike; humans have Choice</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
           <t>Prior draft — polish TBD</t>
         </is>
+      </c>
+      <c r="K20" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -2005,43 +2072,99 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
+          <t>Bhayanaka Ras – Raktabija &amp; Mahakali</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Stage / Video</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Bhayanaka</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Cosmic battlefield</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Karma, Maya, Raktabija, Maa Kali</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Tandava</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Blood-demon myth → Kali Tandava</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Prior draft — polish TBD</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>VI Coda (prior draft)</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
           <t>Shanta Ras &amp; Grand Finale</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>Shanta</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Full stage</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>Full cast</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>Navras anthem</t>
         </is>
       </c>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>Shiva stills Kali; Maya awakens; Namaste</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr">
+      <c r="J22" s="3" t="inlineStr">
         <is>
           <t>Prior draft — polish TBD</t>
         </is>
+      </c>
+      <c r="K22" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -2055,7 +2178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2087,858 +2210,1285 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Screen: Karma Operations – The Hisaab Kitaab Department</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Act I</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Karma Dev</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>AKV, mortals have outpaced the cosmic order… सृष्टि का चक्र बदल चुका है—हमें कर्म ऑपरेशन्स सेंटर संभालने के लिए तुम्हारी बनाई इस माया की ज़रूरत है।</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Live stage</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>स्वागत है आपका 'Karma Operations' में!</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Karma Dev</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>समय का पहिया चलता रहता है, और उस पहिए की धुरी हूँ मैं—'कर्म'। … मेरे साथ हमेशा चलते हैं मेरे दो साए!</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Karma Dev</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>AnuKool: … Very Cool boy! PratiKool: … Bad boy! Boys, मैं आ रहा हूँ!</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Theme: कर्म... पीछे पड़ा है कर्म... AnuKool and PratiKool sprint in.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Act II</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AnuKool</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>हम आ गए महाराज! मैं हूँ आपका दायाँ हाथ—अनुकूल!</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PratiKool</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>और मैं हूँ प्रतिकूल! … कड़वा सच!</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Karma Dev</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>आबादी इतनी बढ़ चुकी है कि हर सेकंड लाखों नए कर्म दर्ज हो रहे हैं।</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Act III</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PratiKool</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>मेरा तो ओवरटाइम हो रहा है… कलयुग जो ठहरा!</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>AnuKool</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>सुना है उन्होंने 'आर्टिफिशियल इंटेलिजेंस' तैयार किया है!</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Karma Dev</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>इस शहर में एक वैज्ञानिक है—AKV। चलो, देखते हैं उसकी उस माया को!</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>AnuKool</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>या या, साइड प्लीज़... Let me swipe and show you!</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>AKV</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Listen, I've created the most advanced humanoid… She has no heart, Karma. She doesn't feel. How are you going to solve that?</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Hey Karma Boys... welcome to our planet! इमॉर्टल्स को पहली बार हम जैसे तुच्छ मॉर्टल्स की ज़रूरत?</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Act IV</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Karma Dev</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Sage Bharat Muni codified the entire human spirit into the Navarasas… we will awaken her artificial neurons through the nine Rasas.</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>अरे, तुम्हें कैसे पता चला साइंटिस्ट?</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>AKV</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>On behalf of humanity, I give this gift back to the immortals. Take Maya with you.</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Narration</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Sanskrit shloka + Hindi narration: love as primal creative impulse</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Karma Dev</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Shringar was easy to compute. The remaining eight Rasas… she will only awaken through an unfolding human story.</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Mother (Shanti)</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>चंदा कब दूर गगन से…</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Bollywood spoof</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Karma Dev</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>ना ना ना… यह तो सिर्फ 'रील लाइफ' का ड्रामा है! असल जिंदगी इससे बिल्कुल अलग होती है।</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Fourth wall</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Shanti</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>भाई! तुम दिन-रात टीवी पर सिर्फ स्पोर्ट्स देखकर अपना वक्त क्यों बर्बाद कर रहे हो?!</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Three Agents</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>हम इन्वेस्टिगेशन ब्यूरो से हैं। हमें आपके भाई की सख्त ज़रूरत है, क्योंकि वे असल में एक सीक्रेट स्पाई हैं। देश की सेवा के लिए हम इन्हें ले जा रहे हैं।</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>IB prank</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Friends</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>करन, तू जब भी मैदान में होता है… Why are you wasting your life behind an office desk? You belong in professional sports!</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Arjun</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>अरे छोड़ो यार… Let him enjoy his riding.</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Defends Karan</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Arjun</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>चल, इन सबको छोड़… एक रेस लगाते हैं!</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Challenge</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Friends</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>सुन अर्जुन… तू अपनी साख का इस्तेमाल करके करन को प्रो-स्पोर्ट्स में स्पॉन्सरशिप क्यों नहीं दिलाता?</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Arjun</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>ठीक है। मेरा एक दोस्त है NEKI में—अजय वालिया। He is a brilliant businessman. मैं उससे बात करता हूँ।</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>NEKI = Ajay Walia's company (Nike parody)</t>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>माया बता देती है!</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Friends / Arjun</t>
+          <t>PratiKool</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>NEKI — नेकी और पूछ-पूछ!</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Brand gag; NEKI rhymes with Hindi नेकी</t>
+          <t>तुम्हारी नहीं, तुम्हारी इस क्रिएशन की ज़रूरत है! Because of your overpopulation!</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Ajay Walia</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>NEKI — नेकी और पूछ-पूछ! सिर्फ टैलेंट से स्पॉन्सरशिप नहीं मिलती। मैं जल्द ही एक बड़ी साइकल रेस स्पॉन्सर कर रहा हूँ—उसमें हिस्सा लो और मुझे अपनी काबिलियत साबित करके दिखाओ।</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>NEKI brand gag + race-to-prove</t>
+      <c r="A18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>AnuKool</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>तो हमें आपकी माया चाहिए to run our Karma Operations!</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Arjun</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>सुन, मैंने तेरे पीछे अपना पूरा नाम और साख दांव पर लगा दी है… पर मुझे पता है, तू यह कर दिखाएगा।</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr"/>
+      <c r="A19" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Maya</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>I love travelling AKV, but this is too far... and I am not sure what's my scope.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Act V</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="A20" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>AKV</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Karma Operations runs on actions, thoughts, and emotions. इसने इमोशन नहीं सीखा है अभी तक!</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>AnuKool</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Don't worry जी, Karma Dev will teach her!</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PratiKool</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>क्या teach her, teach her! मुझे तो शक है कि हमारी जॉब ही खा जाएगी एक दिन!</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" t="inlineStr">
         <is>
           <t>Karma Dev</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>लगता है हमें अपनी कहानी का असली प्लॉट मिल गया है!</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Pratikool</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>लगता है बहुत जल्द आपकी यह नौकरी जाने वाली है, कोच साहब!</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Coach Satak Singh</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>क्या?! क्यों जाएगी मेरी नौकरी?</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Pratikool</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>हम आपके लिए जासूस बनेंगे। वे दोनों पीठ पीछे क्या कर रहे हैं, इसकी पल-पल की खबर हम आपको लाकर देंगे।</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>अब से यह हमारी रिस्पॉन्सिबिलिटी है। हम सिखाएंगे! ...चलो माया, let's go!</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Coach Satak Singh</t>
+          <t>AKV</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>बहुत बढ़िया करन! फॉर्म बिल्कुल सही है, इसी पेस को बनाए रखो।</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Praises Karan</t>
+          <t>Bye Maya, keep in touch!</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Blackout → NAVARASA title song + chariot → screen back to Hisaab Kitaab.</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>→ Scene 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Narration</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Sanskrit shloka + Hindi narration: love as primal creative impulse</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Karma Dev</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Shringar was easy to compute. The remaining eight Rasas… she will only awaken through an unfolding human story.</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Mother (Shanti)</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>चंदा कब दूर गगन से…</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Bollywood spoof</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Karma Dev</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>ना ना ना… यह तो सिर्फ 'रील लाइफ' का ड्रामा है! असल जिंदगी इससे बिल्कुल अलग होती है।</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Fourth wall</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Shanti</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>भाई! तुम दिन-रात टीवी पर सिर्फ स्पोर्ट्स देखकर अपना वक्त क्यों बर्बाद कर रहे हो?!</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Three Agents</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>हम इन्वेस्टिगेशन ब्यूरो से हैं। हमें आपके भाई की सख्त ज़रूरत है, क्योंकि वे असल में एक सीक्रेट स्पाई हैं। देश की सेवा के लिए हम इन्हें ले जा रहे हैं।</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>IB prank</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>करन, तू जब भी मैदान में होता है… Why are you wasting your life behind an office desk? You belong in professional sports!</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
           <t>Arjun</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>देख भाई, ऐसे करते हैं! तू खुद को प्रो एथलीट कहता है ना? असली फॉर्म और स्वैग इसे कहते हैं!</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Showboat + insult</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>10</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Karan uneasy / disappointed in front of others — silent sting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>10</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Pratikool</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>अर्जुन ने दोस्त बनके तुझे मौका दिया—इसका मतलब यह नहीं कि अब वो तेरा मालिक है… जो मर्ज़ी कमांड करे, जो मर्ज़ी बोले!</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Stokes Karan</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>10</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Coach Satak Singh</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>भाई… ये ठीक नहीं हो रहा है।</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Concerned</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>10</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Cool</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>रेस का मार्केटिंग प्री-इवेंट पार्टी है… लेट्स डू सम गुड पार्टी एंड ब्रिंग देयर फ्रेंडशिप बैक।</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Party plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>11</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Maya</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>कर्मा देव… स्टोरी में अचानक ट्विस्ट क्यों आ गया? वे इतने अच्छे दोस्त थे—फिर ये क्या हो रहा है?</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Asks about twist</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>11</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Karma Dev</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>तू भावनाओं के बहुत सारे बदलाव देखने वाली है… और भावनाओं के वे पहलू भी, जो काबू में नहीं रहते। अब उस लर्निंग के लिए तैयार हो जा—पर पहले आसान से शुरू करते हैं। थोड़ा एंटरटेनमेंट… सुना है मार्केटिंग इवेंट है। थोड़ा हँसी-मज़ाक होगा… और मैं तुझे हास्य रस भी सिखा सकता हूँ—जो इंसान की ज़िंदगी के सारे एंटरटेनमेंट की बुनियाद है।</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Hasya setup</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>11</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Maya</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>ओह… हँसी-मज़ाक?</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>11</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Karma Dev</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>(sings Hasya Sanskrit shloka)</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Hasya shloka</t>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>अरे छोड़ो यार… Let him enjoy his riding.</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Defends Karan</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="n">
-        <v>12</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Ruchi</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>(Emcee opens the marketing pre-event party — brings on Arjun)</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Hosts</t>
+      <c r="A34" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Arjun</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>चल, इन सबको छोड़… एक रेस लगाते हैं!</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Challenge</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="n">
-        <v>12</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Comic Qawwali + shayari → Oiyamma → Sharara → Ghaghra slapstick → Dhurandhar</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Hasya medley</t>
-        </is>
-      </c>
+      <c r="A35" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Friends</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>सुन अर्जुन… तू अपनी साख का इस्तेमाल करके करन को प्रो-स्पोर्ट्स में स्पॉन्सरशिप क्यों नहीं दिलाता?</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Pratikool</t>
+          <t>Arjun</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>यह बर्दाश्त मत करना! तूने इस लड़के के लिए अपनी साख दांव पर लगाई, और इसने तेरे ही स्टेज पर आकर तेरी धज्जियां उड़ा दीं!</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr"/>
+          <t>ठीक है। मेरा एक दोस्त है NEKI में—अजय वालिया। He is a brilliant businessman. मैं उससे बात करता हूँ।</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>NEKI = Ajay Walia's company (Nike parody)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="n">
-        <v>13</v>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>Arjun</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>इसने मुझे मेरे ही स्टेज पर नीचा दिखाया है ना? अब मैं इसे कहीं और नहीं, उसी के मैदान में धूल चटाऊँगा! I am going to take him down in his own domain!</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>Dark band</t>
+      <c r="A37" t="n">
+        <v>6</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Friends / Arjun</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>NEKI — नेकी और पूछ-पूछ!</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Brand gag; NEKI rhymes with Hindi नेकी</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Direction</t>
+          <t>Ajay Walia</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Invisible wire across highway; Karan crashes; cycle destroyed; Karma mourning shloka</t>
+          <t>NEKI — नेकी और पूछ-पूछ! सिर्फ टैलेंट से स्पॉन्सरशिप नहीं मिलती। मैं जल्द ही एक बड़ी साइकल रेस स्पॉन्सर कर रहा हूँ—उसमें हिस्सा लो और मुझे अपनी काबिलियत साबित करके दिखाओ।</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Sabotage</t>
+          <t>NEKI brand gag + race-to-prove</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Coach Satak Singh</t>
+          <t>Arjun</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>वालिया साहब, करन का बहुत भयानक एक्सीडेंट हो गया है। साइकल टूट चुकी है और वह खुद चलने की हालत में भी नहीं है।</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
+          <t>सुन, मैंने तेरे पीछे अपना पूरा नाम और साख दांव पर लगा दी है… पर मुझे पता है, तू यह कर दिखाएगा।</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>Ajay Walia</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>नो रिजल्ट्स, नो स्पॉन्सरशिप। तुरंत कॉन्ट्रैक्ट कैंसिल करो!</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>Speakerphone</t>
+      <c r="A40" t="n">
+        <v>8</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Karan singing/dancing last para; Arjun walks in.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>≈3 min</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>Coach Satak Singh</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>करन, तुम्हारी इस हालत के बाद स्पॉन्सरशिप का सवाल ही नहीं उठता। यू कैन नॉट पार्टिसिपेट।</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>Tears contract</t>
+      <c r="A41" t="n">
+        <v>8</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Arjun</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>भाई — बहुत कुछ दाव पर लगाया है मैंने… please focus कर। तेरा परफॉर्मेंस तो मुझसे भी खराब हो रहा है!!!</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="B42" s="3" t="inlineStr">
+      <c r="A42" t="n">
+        <v>8</v>
+      </c>
+      <c r="B42" t="inlineStr">
         <is>
           <t>Karan</t>
         </is>
       </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>मैं अर्जुन को नहीं छोड़ूँगा! उसने धोखे से मुझे गिराया है, आई एम गोइंग टू डिस्ट्रॉय हिम!</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>Bat</t>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>चिल यार, देख लेंगे… साइकल तो बाएँ हाथ का खेल है…</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Hand on shoulder</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>Cool</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>करन, रुक! बदले की आग में सिर्फ तू खुद को जलाएगा। असली जवाब अर्जुन को तोड़ना नहीं, मैदान में वापस खड़ा होकर दिखाना है!</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr"/>
+      <c r="A43" t="n">
+        <v>8</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Arjun</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>अजय वालिया ने तो धमकी दी है… मेरे और कोच का भी लाइफ बर्बाद कर देगा…</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>Brishti</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>गुस्सा छोड़ करन। पहले फिजियोथेरेपी शुरू करते हैं, तुम्हारी चोटों को हील करना पहली प्रायोरिटी है।</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr"/>
+      <c r="A44" t="n">
+        <v>8</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Karan</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>अरे कुछ नहीं होगा… कोच सतक सिंह के साथ तो मस्त कॉमेडी होने वाला है…</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="n">
-        <v>16</v>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>Gaurav</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>वालिया ने स्पॉन्सरशिप छीनी है ना? तेरी हिम्मत कोई नहीं छीन सकता। We are going to fund and back you!</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr"/>
+      <c r="A45" t="n">
+        <v>8</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Arjun</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>बाएँ हाथ नहीं — पैर से चलाना पड़ेगा।</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Both laugh</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Anu</t>
+          <t>Karma Dev</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>डाइट, रिकवरी और स्ट्रेंथ ट्रेनिंग का नया प्लान मैं बना रही हूँ। एक-एक दिन का हिसाब रखेंगे।</t>
+          <t>लगता है हमें अपनी कहानी का असली प्लॉट मिल गया है!</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Shikha</t>
+          <t>PratiKool</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>और उस टूटी हुई साइकल की चिंता मत कर। जब तक तू खड़ा होगा, तेरी बाइक पहले से ज्यादा तेज दौड़ने के लिए तैयार मिलेगी!</t>
+          <t>लगता है बहुत जल्द आपकी यह नौकरी जाने वाली है, कोच साहब!</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Coach Satak Singh</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>क्या?! क्यों जाएगी मेरी नौकरी?</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>PratiKool</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>हम आपके लिए जासूस बनेंगे। वे दोनों पीठ पीछे क्या कर रहे हैं, इसकी पल-पल की खबर हम आपको लाकर देंगे।</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>11</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Coach Satak Singh</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>बहुत बढ़िया करन! फॉर्म बिल्कुल सही है, इसी पेस को बनाए रखो।</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Praises Karan</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>11</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Arjun</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>देख भाई, ऐसे करते हैं! तू खुद को प्रो एथलीट कहता है ना? असली फॉर्म और स्वैग इसे कहते हैं!</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Showboat + insult</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>11</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Karan uneasy / disappointed in front of others — silent sting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>11</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>PratiKool</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>अर्जुन ने दोस्त बनके तुझे मौका दिया—इसका मतलब यह नहीं कि अब वो तेरा मालिक है… जो मर्ज़ी कमांड करे, जो मर्ज़ी बोले!</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Stokes Karan</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>11</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Coach Satak Singh</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>भाई… ये ठीक नहीं हो रहा है।</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Concerned</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>11</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>AnuKool</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>रेस का मार्केटिंग प्री-इवेंट पार्टी है… लेट्स डू सम गुड पार्टी एंड ब्रिंग देयर फ्रेंडशिप बैक।</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Party plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>12</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Maya</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>कर्मा देव… स्टोरी में अचानक ट्विस्ट क्यों आ गया? वे इतने अच्छे दोस्त थे—फिर ये क्या हो रहा है?</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Asks about twist</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>12</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Karma Dev</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>तू भावनाओं के बहुत सारे बदलाव देखने वाली है… और भावनाओं के वे पहलू भी, जो काबू में नहीं रहते। अब उस लर्निंग के लिए तैयार हो जा—पर पहले आसान से शुरू करते हैं। थोड़ा एंटरटेनमेंट… सुना है मार्केटिंग इवेंट है। थोड़ा हँसी-मज़ाक होगा… और मैं तुझे हास्य रस भी सिखा सकता हूँ—जो इंसान की ज़िंदगी के सारे एंटरटेनमेंट की बुनियाद है।</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Hasya setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>12</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Maya</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>ओह… हँसी-मज़ाक?</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>12</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Karma Dev</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>(sings Hasya Sanskrit shloka)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Hasya shloka</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>13</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Ruchi</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>(Emcee opens the marketing pre-event party — brings on Arjun)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Hosts</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>13</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Comic Qawwali + shayari → Oiyamma → Sharara → Ghaghra slapstick → Dhurandhar</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Hasya medley</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>PratiKool</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>यह बर्दाश्त मत करना! तूने इस लड़के के लिए अपनी साख दांव पर लगाई, और इसने तेरे ही स्टेज पर आकर तेरी धज्जियां उड़ा दीं!</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Arjun</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>इसने मुझे मेरे ही स्टेज पर नीचा दिखाया है ना? अब मैं इसे कहीं और नहीं, उसी के मैदान में धूल चटाऊँगा! I am going to take him down in his own domain!</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Dark band</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Invisible wire across highway; Karan crashes; cycle destroyed; Karma mourning shloka</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Sabotage</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="B48" s="3" t="inlineStr">
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Coach Satak Singh</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>वालिया साहब, करन का बहुत भयानक एक्सीडेंट हो गया है। साइकल टूट चुकी है और वह खुद चलने की हालत में भी नहीं है।</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Ajay Walia</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>नो रिजल्ट्स, नो स्पॉन्सरशिप। तुरंत कॉन्ट्रैक्ट कैंसिल करो!</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Speakerphone</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Coach Satak Singh</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>करन, तुम्हारी इस हालत के बाद स्पॉन्सरशिप का सवाल ही नहीं उठता। यू कैन नॉट पार्टिसिपेट।</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Tears contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Karan</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>मैं अर्जुन को नहीं छोड़ूँगा! उसने धोखे से मुझे गिराया है, आई एम गोइंग टू डिस्ट्रॉय हिम!</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Bat</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>AnuKool</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>करन, रुक! बदले की आग में सिर्फ तू खुद को जलाएगा। असली जवाब अर्जुन को तोड़ना नहीं, मैदान में वापस खड़ा होकर दिखाना है!</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Brishti</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>गुस्सा छोड़ करन। पहले फिजियोथेरेपी शुरू करते हैं, तुम्हारी चोटों को हील करना पहली प्रायोरिटी है।</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Gaurav</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>वालिया ने स्पॉन्सरशिप छीनी है ना? तेरी हिम्मत कोई नहीं छीन सकता। We are going to fund and back you!</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Anu</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>डाइट, रिकवरी और स्ट्रेंथ ट्रेनिंग का नया प्लान मैं बना रही हूँ। एक-एक दिन का हिसाब रखेंगे।</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Shikha</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>और उस टूटी हुई साइकल की चिंता मत कर। जब तक तू खड़ा होगा, तेरी बाइक पहले से ज्यादा तेज दौड़ने के लिए तैयार मिलेगी!</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
         <is>
           <t>Shri</t>
         </is>
       </c>
-      <c r="C48" s="3" t="inlineStr">
+      <c r="C74" s="3" t="inlineStr">
         <is>
           <t>हम सब तेरे साथ हैं करन। तुझे बस अपनी नजर फिनिश लाइन पर रखनी है।</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr"/>
+      <c r="D74" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2951,7 +3501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2988,7 +3538,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Futuristic entrance theme</t>
+          <t>Ethereal welcome + कर्म... पीछे पड़ा है कर्म</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2998,7 +3548,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AKV + Maya step from screen</t>
+          <t>AnuKool &amp; PratiKool sprint in</t>
         </is>
       </c>
     </row>
@@ -3008,7 +3558,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Navras / Karma Chakra title anthem</t>
+          <t>NAVARASA title song / Karma Chakra</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3018,7 +3568,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Chariot ascent</t>
+          <t>Exit back to Hisaab Kitaab</t>
         </is>
       </c>
     </row>
@@ -3184,7 +3734,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -3204,7 +3754,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -3224,7 +3774,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -3244,7 +3794,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -3264,7 +3814,7 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -3284,7 +3834,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -3304,7 +3854,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -3324,7 +3874,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -3344,7 +3894,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -3364,7 +3914,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -3384,7 +3934,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -3404,7 +3954,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -3424,7 +3974,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -3444,7 +3994,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -3464,7 +4014,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -3484,7 +4034,7 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -3504,7 +4054,7 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -3519,6 +4069,46 @@
       <c r="D28" t="inlineStr">
         <is>
           <t>Prior draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>1</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Maya theme</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Reveal</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>AnuKool swipe → AKV lab</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>8</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Celebration / song last para coda</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Live stage</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Karan sings; Arjun interruption</t>
         </is>
       </c>
     </row>
@@ -3533,7 +4123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3598,7 +4188,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Lab set TBD</t>
+          <t>Karma Ops screen + tech hub</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -3613,7 +4203,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Screen-to-stage handoff; chariot</t>
+          <t>Hisaab Kitaab welcome; shadow entrance; Maya handover</t>
         </is>
       </c>
     </row>
@@ -3828,37 +4418,37 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Screen → Stage</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>Yes (AI trails)</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Stage — song coda</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Descent graphic</t>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>≈3 min · focus / Walia beat</t>
         </is>
       </c>
     </row>
@@ -3868,7 +4458,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>Screen → Stage</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -3878,12 +4468,12 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Camp</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (AI trails)</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -3893,7 +4483,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Spy hire</t>
+          <t>Descent graphic</t>
         </is>
       </c>
     </row>
@@ -3913,12 +4503,12 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Gym</t>
+          <t>Camp</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -3928,7 +4518,7 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Pratikool sting + Cool party pitch</t>
+          <t>Spy hire</t>
         </is>
       </c>
     </row>
@@ -3938,102 +4528,102 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Gym</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>PratiKool sting + AnuKool party pitch</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
           <t>Video / Stage</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Karma Ops Center</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Hasya setup + shloka</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>TBD — assign</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Marketing pre-event party</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>Qawwali + medley</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>TBD — clash</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Stage</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Malhari clash mid-party</t>
         </is>
       </c>
     </row>
@@ -4043,32 +4633,32 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Video</t>
+          <t>Stage</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TBD — clash</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Highway</t>
+          <t>Stage</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Wire gag + crash VFX</t>
+          <t>Malhari clash mid-party</t>
         </is>
       </c>
     </row>
@@ -4078,7 +4668,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Video / Stage</t>
+          <t>Video</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -4088,7 +4678,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Hospital</t>
+          <t>Highway</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -4098,12 +4688,12 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Contract tear slow-mo</t>
+          <t>Wire gag + crash VFX</t>
         </is>
       </c>
     </row>
@@ -4113,30 +4703,65 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
+          <t>Video / Stage</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Contract tear slow-mo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
           <t>Stage → Montage</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Ward / garage / track</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Yes (montage)</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Friend role lines</t>
         </is>
@@ -4226,7 +4851,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>11–12</t>
+          <t>12–13</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -4251,7 +4876,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -4276,7 +4901,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>14 (lead-in)</t>
+          <t>15 (lead-in)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -4301,7 +4926,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -4326,7 +4951,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -4351,7 +4976,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -4376,7 +5001,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -4401,7 +5026,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">

</xml_diff>